<commit_message>
test: all v2.0.0 features tested and working
</commit_message>
<xml_diff>
--- a/media/reports/RPL/laporan_RPL_2026_03.xlsx
+++ b/media/reports/RPL/laporan_RPL_2026_03.xlsx
@@ -8,7 +8,6 @@
   </bookViews>
   <sheets>
     <sheet name="Semua Kelas" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="XII RPL" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -67,7 +66,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
@@ -75,10 +74,6 @@
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -444,18 +439,18 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J4"/>
+  <dimension ref="A1:J3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
     <col width="6" customWidth="1" min="2" max="2"/>
-    <col width="19" customWidth="1" min="3" max="3"/>
-    <col width="12" customWidth="1" min="4" max="4"/>
-    <col width="8" customWidth="1" min="5" max="5"/>
+    <col width="7" customWidth="1" min="3" max="3"/>
+    <col width="8" customWidth="1" min="4" max="4"/>
+    <col width="7" customWidth="1" min="5" max="5"/>
     <col width="9" customWidth="1" min="6" max="6"/>
     <col width="13" customWidth="1" min="7" max="7"/>
     <col width="14" customWidth="1" min="8" max="8"/>
-    <col width="12" customWidth="1" min="9" max="9"/>
+    <col width="9" customWidth="1" min="9" max="9"/>
     <col width="8" customWidth="1" min="10" max="10"/>
   </cols>
   <sheetData>
@@ -515,190 +510,6 @@
       <c r="J3" s="2" t="inlineStr">
         <is>
           <t>Denda</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="3" t="n">
-        <v>1</v>
-      </c>
-      <c r="B4" s="3" t="inlineStr">
-        <is>
-          <t>999</t>
-        </is>
-      </c>
-      <c r="C4" s="4" t="inlineStr">
-        <is>
-          <t>Peminjam Laporan</t>
-        </is>
-      </c>
-      <c r="D4" s="3" t="inlineStr">
-        <is>
-          <t>XII RPL A</t>
-        </is>
-      </c>
-      <c r="E4" s="4" t="inlineStr">
-        <is>
-          <t>Obeng</t>
-        </is>
-      </c>
-      <c r="F4" s="3" t="n">
-        <v>1</v>
-      </c>
-      <c r="G4" s="3" t="inlineStr">
-        <is>
-          <t>14/03/2026</t>
-        </is>
-      </c>
-      <c r="H4" s="3" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="I4" s="3" t="inlineStr">
-        <is>
-          <t>Disetujui</t>
-        </is>
-      </c>
-      <c r="J4" s="4" t="inlineStr">
-        <is>
-          <t>Rp0</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <mergeCells count="1">
-    <mergeCell ref="A1:J1"/>
-  </mergeCells>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:J4"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="5" customWidth="1" min="1" max="1"/>
-    <col width="6" customWidth="1" min="2" max="2"/>
-    <col width="19" customWidth="1" min="3" max="3"/>
-    <col width="12" customWidth="1" min="4" max="4"/>
-    <col width="8" customWidth="1" min="5" max="5"/>
-    <col width="9" customWidth="1" min="6" max="6"/>
-    <col width="13" customWidth="1" min="7" max="7"/>
-    <col width="14" customWidth="1" min="8" max="8"/>
-    <col width="12" customWidth="1" min="9" max="9"/>
-    <col width="8" customWidth="1" min="10" max="10"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>LAPORAN PEMINJAMAN - XII RPL</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="2" t="inlineStr">
-        <is>
-          <t>No</t>
-        </is>
-      </c>
-      <c r="B3" s="2" t="inlineStr">
-        <is>
-          <t>NIS</t>
-        </is>
-      </c>
-      <c r="C3" s="2" t="inlineStr">
-        <is>
-          <t>Nama</t>
-        </is>
-      </c>
-      <c r="D3" s="2" t="inlineStr">
-        <is>
-          <t>Kelas</t>
-        </is>
-      </c>
-      <c r="E3" s="2" t="inlineStr">
-        <is>
-          <t>Alat</t>
-        </is>
-      </c>
-      <c r="F3" s="2" t="inlineStr">
-        <is>
-          <t>Jumlah</t>
-        </is>
-      </c>
-      <c r="G3" s="2" t="inlineStr">
-        <is>
-          <t>Tgl Pinjam</t>
-        </is>
-      </c>
-      <c r="H3" s="2" t="inlineStr">
-        <is>
-          <t>Tgl Kembali</t>
-        </is>
-      </c>
-      <c r="I3" s="2" t="inlineStr">
-        <is>
-          <t>Status</t>
-        </is>
-      </c>
-      <c r="J3" s="2" t="inlineStr">
-        <is>
-          <t>Denda</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="3" t="n">
-        <v>1</v>
-      </c>
-      <c r="B4" s="3" t="inlineStr">
-        <is>
-          <t>999</t>
-        </is>
-      </c>
-      <c r="C4" s="4" t="inlineStr">
-        <is>
-          <t>Peminjam Laporan</t>
-        </is>
-      </c>
-      <c r="D4" s="3" t="inlineStr">
-        <is>
-          <t>XII RPL A</t>
-        </is>
-      </c>
-      <c r="E4" s="4" t="inlineStr">
-        <is>
-          <t>Obeng</t>
-        </is>
-      </c>
-      <c r="F4" s="3" t="n">
-        <v>1</v>
-      </c>
-      <c r="G4" s="3" t="inlineStr">
-        <is>
-          <t>14/03/2026</t>
-        </is>
-      </c>
-      <c r="H4" s="3" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="I4" s="3" t="inlineStr">
-        <is>
-          <t>Disetujui</t>
-        </is>
-      </c>
-      <c r="J4" s="4" t="inlineStr">
-        <is>
-          <t>Rp0</t>
         </is>
       </c>
     </row>

</xml_diff>